<commit_message>
- Enhance POS Automation Reporting and Logging
- Added new HTML reports for POS automation runs with detailed execution, performance, stability, and failure summaries.
- Updated the batch script to conditionally open the live dashboard based on configuration settings.
- Modified configuration settings to adjust duration and product details for the automation runs.
- Refactored state detection logic in BasePage to improve accuracy in identifying the POS menu.
- Implemented a new run artifacts utility to manage logging and report generation directories.
- Enhanced logging functionality to include file logging for better traceability of automation runs.
- Updated ADB utility functions to improve stability during automation sessions.
- Adjusted Excel and HTML report generation to utilize the new run artifacts directory structure.
</commit_message>
<xml_diff>
--- a/Analytics/reports/report.xlsx
+++ b/Analytics/reports/report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="49">
   <si>
     <t>Cycle</t>
   </si>
@@ -29,12 +29,93 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>10000 ms</t>
+    <t>9439 ms</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
+    <t>7532 ms</t>
+  </si>
+  <si>
+    <t>7583 ms</t>
+  </si>
+  <si>
+    <t>7683 ms</t>
+  </si>
+  <si>
+    <t>8115 ms</t>
+  </si>
+  <si>
+    <t>8499 ms</t>
+  </si>
+  <si>
+    <t>7968 ms</t>
+  </si>
+  <si>
+    <t>7334 ms</t>
+  </si>
+  <si>
+    <t>8655 ms</t>
+  </si>
+  <si>
+    <t>7916 ms</t>
+  </si>
+  <si>
+    <t>7298 ms</t>
+  </si>
+  <si>
+    <t>7665 ms</t>
+  </si>
+  <si>
+    <t>7253 ms</t>
+  </si>
+  <si>
+    <t>8749 ms</t>
+  </si>
+  <si>
+    <t>7180 ms</t>
+  </si>
+  <si>
+    <t>7434 ms</t>
+  </si>
+  <si>
+    <t>7318 ms</t>
+  </si>
+  <si>
+    <t>6915 ms</t>
+  </si>
+  <si>
+    <t>7716 ms</t>
+  </si>
+  <si>
+    <t>7365 ms</t>
+  </si>
+  <si>
+    <t>8635 ms</t>
+  </si>
+  <si>
+    <t>7965 ms</t>
+  </si>
+  <si>
+    <t>7368 ms</t>
+  </si>
+  <si>
+    <t>7887 ms</t>
+  </si>
+  <si>
+    <t>7116 ms</t>
+  </si>
+  <si>
+    <t>8382 ms</t>
+  </si>
+  <si>
+    <t>7267 ms</t>
+  </si>
+  <si>
+    <t>7984 ms</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -56,7 +137,7 @@
     <t>Orders Per Minute</t>
   </si>
   <si>
-    <t>6.0</t>
+    <t>8.3</t>
   </si>
   <si>
     <t>Recoveries</t>
@@ -71,7 +152,7 @@
     <t>Slowdown Percent</t>
   </si>
   <si>
-    <t>0%</t>
+    <t>-2.8%</t>
   </si>
   <si>
     <t>Memory Leak Indicator</t>
@@ -481,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -514,6 +595,426 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>33</v>
+      </c>
+      <c r="D31" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" t="s">
         <v>6</v>
       </c>
     </row>
@@ -534,39 +1035,39 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="B5" s="4">
         <v>0</v>
@@ -574,15 +1075,15 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>6</v>
@@ -590,15 +1091,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>6</v>
@@ -606,7 +1107,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>6</v>

</xml_diff>